<commit_message>
refactor: remove orphanPolicy handling from import process and update documentation
</commit_message>
<xml_diff>
--- a/tests/fixtures/pedidos.xlsx
+++ b/tests/fixtures/pedidos.xlsx
@@ -396,7 +396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -430,17 +430,6 @@
       </c>
       <c r="C3">
         <v>89.9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>103</v>
-      </c>
-      <c r="B4">
-        <v>999</v>
-      </c>
-      <c r="C4">
-        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add produto field to pedidos and update related functionality
</commit_message>
<xml_diff>
--- a/tests/fixtures/pedidos.xlsx
+++ b/tests/fixtures/pedidos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>id</t>
   </si>
@@ -20,6 +20,15 @@
   </si>
   <si>
     <t>valor</t>
+  </si>
+  <si>
+    <t>produto</t>
+  </si>
+  <si>
+    <t>Notebook</t>
+  </si>
+  <si>
+    <t>Mouse</t>
   </si>
 </sst>
 </file>
@@ -396,10 +405,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -409,8 +418,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>101</v>
       </c>
@@ -420,8 +432,11 @@
       <c r="C2">
         <v>150.5</v>
       </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>102</v>
       </c>
@@ -430,6 +445,9 @@
       </c>
       <c r="C3">
         <v>89.9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>